<commit_message>
Updates to Config Files
Added dummy data to config files, updated config files to EV LIB format
</commit_message>
<xml_diff>
--- a/docs/Files/ODYM_Config_Tutorial6_LIB.xlsx
+++ b/docs/Files/ODYM_Config_Tutorial6_LIB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elanphear\Code\ODYM\docs\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E57BB31-2221-4CE5-8C60-1188E3F5ED97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120950A2-5D3B-4B47-BAA0-2C625E0A920B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="5" r:id="rId1"/>
@@ -995,14 +995,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5546875" customWidth="1"/>
+    <col min="4" max="4" width="26.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B1" s="29" t="s">
         <v>37</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="6"/>
       <c r="B2" s="8" t="s">
         <v>38</v>
@@ -1020,12 +1020,12 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="6"/>
       <c r="B3" s="8"/>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="6"/>
       <c r="B4" s="9" t="s">
         <v>2</v>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="G4" s="35"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="6"/>
       <c r="B5" s="9" t="s">
         <v>51</v>
@@ -1050,122 +1050,122 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="6"/>
       <c r="B6" s="9"/>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="6"/>
       <c r="B7" s="9"/>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="6"/>
       <c r="B8" s="9"/>
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="6"/>
       <c r="B9" s="11"/>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="10"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="10"/>
       <c r="B11" s="12"/>
       <c r="C11" s="14"/>
       <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="10"/>
       <c r="B12" s="12"/>
       <c r="C12" s="15"/>
       <c r="D12" s="12"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="10"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="10"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="10"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="10"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="10"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="10"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="10"/>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="10"/>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="10"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="10"/>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="6"/>
       <c r="B25" s="1"/>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="1"/>
       <c r="C26" s="2"/>
@@ -1179,19 +1179,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:J59"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="4.88671875" customWidth="1"/>
+    <col min="2" max="2" width="4.90625" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="44.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.6640625" customWidth="1"/>
-    <col min="6" max="6" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6328125" customWidth="1"/>
+    <col min="6" max="6" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.36328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B2" s="18" t="s">
         <v>3</v>
       </c>
@@ -1202,7 +1202,7 @@
       <c r="G2" s="19"/>
       <c r="H2" s="20"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C3" s="23" t="s">
         <v>27</v>
       </c>
@@ -1214,7 +1214,7 @@
       <c r="G3" s="30"/>
       <c r="H3" s="30"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>4</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>0</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>5</v>
       </c>
@@ -1238,11 +1238,11 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D7" s="7"/>
       <c r="J7" s="13"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B8" s="18" t="s">
         <v>39</v>
       </c>
@@ -1254,7 +1254,7 @@
       <c r="H8" s="20"/>
       <c r="J8" s="13"/>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C9" s="23" t="s">
         <v>27</v>
       </c>
@@ -1269,7 +1269,7 @@
       <c r="H9" s="30"/>
       <c r="J9" s="13"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>6</v>
       </c>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="J10" s="13"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>56</v>
       </c>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="J11" s="13"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>57</v>
       </c>
@@ -1296,10 +1296,10 @@
       </c>
       <c r="J12" s="13"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.35">
       <c r="J13" s="17"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>49</v>
       </c>
@@ -1312,7 +1312,7 @@
       <c r="G14" s="19"/>
       <c r="H14" s="20"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C15" s="24" t="s">
         <v>7</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C16" s="25" t="s">
         <v>11</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C17" s="25" t="s">
         <v>71</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C18" s="25" t="s">
         <v>15</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C19" s="25" t="s">
         <v>16</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C20" s="25" t="s">
         <v>77</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C21" s="25" t="s">
         <v>59</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C22" s="25" t="s">
         <v>12</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C23" s="25" t="s">
         <v>14</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C24" s="21" t="s">
         <v>86</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>45</v>
       </c>
@@ -1556,7 +1556,7 @@
       <c r="G26" s="19"/>
       <c r="H26" s="20"/>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C27" s="26" t="s">
         <v>46</v>
       </c>
@@ -1572,7 +1572,7 @@
       <c r="G27" s="30"/>
       <c r="H27" s="30"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C28" s="31">
         <v>0</v>
       </c>
@@ -1586,7 +1586,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C29" s="31">
         <v>1</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C30" s="27">
         <v>2</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C31" s="27">
         <v>3</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C32" s="31">
         <v>4</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C33" s="27">
         <v>5</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C34" s="31">
         <v>6</v>
       </c>
@@ -1655,7 +1655,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C35" s="27">
         <v>7</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C36" s="31">
         <v>8</v>
       </c>
@@ -1677,7 +1677,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B38" s="18" t="s">
         <v>25</v>
       </c>
@@ -1688,7 +1688,7 @@
       <c r="G38" s="19"/>
       <c r="H38" s="20"/>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C39" s="26" t="s">
         <v>28</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C40" t="s">
         <v>92</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C41" s="27" t="s">
         <v>95</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C42" s="27" t="s">
         <v>96</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C43" s="27" t="s">
         <v>103</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C44" s="27" t="s">
         <v>106</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C45" s="27" t="s">
         <v>105</v>
       </c>
@@ -1846,10 +1846,10 @@
         <v>110</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C46" s="27"/>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B47" s="18" t="s">
         <v>40</v>
       </c>
@@ -1860,12 +1860,12 @@
       <c r="G47" s="19"/>
       <c r="H47" s="20"/>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C48" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C49" s="27" t="s">
         <v>42</v>
       </c>
@@ -1876,22 +1876,22 @@
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.35">
       <c r="D50" s="33"/>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.35">
       <c r="D51" s="33"/>
     </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.35">
       <c r="D52" s="33"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.35">
       <c r="D53" s="33"/>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.35">
       <c r="D54" s="33"/>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B56" s="18" t="s">
         <v>48</v>
       </c>
@@ -1902,12 +1902,12 @@
       <c r="G56" s="19"/>
       <c r="H56" s="20"/>
     </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C57" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B59" s="18" t="s">
         <v>112</v>
       </c>

</xml_diff>